<commit_message>
Daily NIFTY valuation update
</commit_message>
<xml_diff>
--- a/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
+++ b/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backtest" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth_Matrix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal_Backtest" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly_Data" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PE_History_Post2021" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Log" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Backtest" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Growth_Matrix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Signal_Backtest" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Quarterly_Data" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PE_History_Post2021" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Daily_Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Methodology" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Quarterly_Data'!$A$4:$R$114</definedName>
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;[Red](#,##0.00);-"/>
     <numFmt numFmtId="166" formatCode="0.00x;[Red](0.00x);-"/>
@@ -34,6 +34,9 @@
     <numFmt numFmtId="168" formatCode="0.0%;[Red](0.0%);-"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
     <numFmt numFmtId="170" formatCode="0.0x;[Red](0.0x);-"/>
+    <numFmt numFmtId="171" formatCode="0.00x"/>
+    <numFmt numFmtId="172" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -102,7 +105,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +147,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -162,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -282,6 +290,14 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -403,13 +419,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -433,7 +449,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -457,7 +473,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -481,7 +497,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -512,8 +528,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -539,8 +555,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -2047,7 +2063,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -2062,9 +2078,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2489,7 +2505,7 @@
         </is>
       </c>
       <c r="B12" s="42" t="n">
-        <v>45930</v>
+        <v>45918</v>
       </c>
     </row>
     <row r="13">
@@ -2499,7 +2515,7 @@
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>24691.95</v>
+        <v>25423.6</v>
       </c>
     </row>
     <row r="14">
@@ -2509,7 +2525,7 @@
         </is>
       </c>
       <c r="B14" s="47" t="n">
-        <v>21.8</v>
+        <v>22.33</v>
       </c>
     </row>
     <row r="15">
@@ -13658,7 +13674,7 @@
       <c r="A70" s="54" t="n">
         <v>46283</v>
       </c>
-      <c r="B70" s="53" t="n">
+      <c r="B70" s="57" t="n">
         <v>19.74</v>
       </c>
       <c r="C70" s="30" t="inlineStr">
@@ -13668,7 +13684,7 @@
       </c>
       <c r="D70" s="34" t="inlineStr">
         <is>
-          <t>https://downstox.com/nifty-pe/nifty-50</t>
+          <t>https://www.nseindia.com/all-reports</t>
         </is>
       </c>
     </row>
@@ -13690,7 +13706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13832,6 +13848,50 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>https://finance.yahoo.com/quote/%5ENSEI/history/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="58" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B6" s="59" t="n">
+        <v>23346.4</v>
+      </c>
+      <c r="C6" s="60" t="n">
+        <v>19.74</v>
+      </c>
+      <c r="D6" s="61" t="n">
+        <v>0.05303030303030303</v>
+      </c>
+      <c r="E6" s="62" t="n">
+        <v>1182.695035460993</v>
+      </c>
+      <c r="F6" s="61" t="n">
+        <v>0.03878208207507883</v>
+      </c>
+      <c r="G6" s="63" t="n">
+        <v>94.6969696969697</v>
+      </c>
+      <c r="H6" s="63" t="n">
+        <v>35.51283283003153</v>
+      </c>
+      <c r="I6" s="63" t="n">
+        <v>76.94172863688824</v>
+      </c>
+      <c r="J6" s="64" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/indices/ind_close_all_18092026.csv</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/indices/ind_close_all_18092026.csv</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NIFTY valuation and backtest update
</commit_message>
<xml_diff>
--- a/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
+++ b/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="B9" s="45">
-        <f>IFERROR((COUNTIF(PE_History_Post2021!$B$5:$B$2000,"&lt;"&amp;B7)+0.5*COUNTIF(PE_History_Post2021!$B$5:$B$2000,B7))/COUNT(PE_History_Post2021!$B$5:$B$2000),"")</f>
+        <f>IFERROR((COUNTIF(PE_History_Post2021!$B$5:$B$500,"&lt;"&amp;B7)+0.5*COUNTIF(PE_History_Post2021!$B$5:$B$500,B7))/COUNT(PE_History_Post2021!$B$5:$B$500),"")</f>
         <v/>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="B10" s="46">
-        <f>IFERROR(MEDIAN(PE_History_Post2021!$B$5:$B$2000),"")</f>
+        <f>MEDIAN(PE_History_Post2021!$B$5:$B$500)</f>
         <v/>
       </c>
       <c r="D10" s="12">
@@ -2913,6 +2913,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3137,6 +3138,8 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -3361,6 +3364,8 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -3585,6 +3590,8 @@
         <v/>
       </c>
     </row>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
@@ -3809,6 +3816,8 @@
         <v/>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
@@ -3863,6 +3872,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3983,6 +3993,7 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
@@ -4191,6 +4202,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
@@ -4326,6 +4338,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4514,6 +4527,8 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -4747,7 +4762,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="n">
+      <c r="A5" s="54" t="n">
         <v>36250</v>
       </c>
       <c r="B5" s="28" t="n">
@@ -4767,7 +4782,7 @@
       </c>
       <c r="F5" s="50" t="inlineStr"/>
       <c r="G5" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C5)+0.5*COUNTIF($C$5:$C$92,C5))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C5)+(COUNTIF($C$5:$C$92,C5)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H5">
@@ -4791,7 +4806,7 @@
         <v/>
       </c>
       <c r="M5">
-        <f>IF(F5="","",IF(F5&lt;5%,"&lt;5%",IF(F5&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F5="","",IF(F5&lt;5%,"&lt;5%",IF(F5&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N5" s="50">
@@ -4816,7 +4831,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="n">
+      <c r="A6" s="54" t="n">
         <v>36341</v>
       </c>
       <c r="B6" s="28" t="n">
@@ -4836,7 +4851,7 @@
       </c>
       <c r="F6" s="50" t="inlineStr"/>
       <c r="G6" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C6)+0.5*COUNTIF($C$5:$C$92,C6))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C6)+(COUNTIF($C$5:$C$92,C6)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H6">
@@ -4860,7 +4875,7 @@
         <v/>
       </c>
       <c r="M6">
-        <f>IF(F6="","",IF(F6&lt;5%,"&lt;5%",IF(F6&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F6="","",IF(F6&lt;5%,"&lt;5%",IF(F6&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N6" s="50">
@@ -4885,7 +4900,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="n">
+      <c r="A7" s="54" t="n">
         <v>36433</v>
       </c>
       <c r="B7" s="28" t="n">
@@ -4905,7 +4920,7 @@
       </c>
       <c r="F7" s="50" t="inlineStr"/>
       <c r="G7" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C7)+0.5*COUNTIF($C$5:$C$92,C7))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C7)+(COUNTIF($C$5:$C$92,C7)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H7">
@@ -4929,7 +4944,7 @@
         <v/>
       </c>
       <c r="M7">
-        <f>IF(F7="","",IF(F7&lt;5%,"&lt;5%",IF(F7&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F7="","",IF(F7&lt;5%,"&lt;5%",IF(F7&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N7" s="50">
@@ -4954,7 +4969,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="n">
+      <c r="A8" s="54" t="n">
         <v>36525</v>
       </c>
       <c r="B8" s="28" t="n">
@@ -4974,7 +4989,7 @@
       </c>
       <c r="F8" s="50" t="inlineStr"/>
       <c r="G8" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C8)+0.5*COUNTIF($C$5:$C$92,C8))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C8)+(COUNTIF($C$5:$C$92,C8)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H8">
@@ -4998,7 +5013,7 @@
         <v/>
       </c>
       <c r="M8">
-        <f>IF(F8="","",IF(F8&lt;5%,"&lt;5%",IF(F8&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F8="","",IF(F8&lt;5%,"&lt;5%",IF(F8&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N8" s="50">
@@ -5023,7 +5038,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="n">
+      <c r="A9" s="54" t="n">
         <v>36616</v>
       </c>
       <c r="B9" s="28" t="n">
@@ -5046,7 +5061,7 @@
         <v/>
       </c>
       <c r="G9" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C9)+0.5*COUNTIF($C$5:$C$92,C9))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C9)+(COUNTIF($C$5:$C$92,C9)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H9">
@@ -5070,7 +5085,7 @@
         <v/>
       </c>
       <c r="M9">
-        <f>IF(F9="","",IF(F9&lt;5%,"&lt;5%",IF(F9&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F9="","",IF(F9&lt;5%,"&lt;5%",IF(F9&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N9" s="50">
@@ -5095,7 +5110,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="n">
+      <c r="A10" s="54" t="n">
         <v>36707</v>
       </c>
       <c r="B10" s="28" t="n">
@@ -5118,7 +5133,7 @@
         <v/>
       </c>
       <c r="G10" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C10)+0.5*COUNTIF($C$5:$C$92,C10))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C10)+(COUNTIF($C$5:$C$92,C10)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H10">
@@ -5142,7 +5157,7 @@
         <v/>
       </c>
       <c r="M10">
-        <f>IF(F10="","",IF(F10&lt;5%,"&lt;5%",IF(F10&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F10="","",IF(F10&lt;5%,"&lt;5%",IF(F10&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N10" s="50">
@@ -5167,7 +5182,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="n">
+      <c r="A11" s="54" t="n">
         <v>36799</v>
       </c>
       <c r="B11" s="28" t="n">
@@ -5190,7 +5205,7 @@
         <v/>
       </c>
       <c r="G11" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C11)+0.5*COUNTIF($C$5:$C$92,C11))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C11)+(COUNTIF($C$5:$C$92,C11)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H11">
@@ -5214,7 +5229,7 @@
         <v/>
       </c>
       <c r="M11">
-        <f>IF(F11="","",IF(F11&lt;5%,"&lt;5%",IF(F11&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F11="","",IF(F11&lt;5%,"&lt;5%",IF(F11&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N11" s="50">
@@ -5239,7 +5254,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="n">
+      <c r="A12" s="54" t="n">
         <v>36891</v>
       </c>
       <c r="B12" s="28" t="n">
@@ -5262,7 +5277,7 @@
         <v/>
       </c>
       <c r="G12" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C12)+0.5*COUNTIF($C$5:$C$92,C12))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C12)+(COUNTIF($C$5:$C$92,C12)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H12">
@@ -5286,7 +5301,7 @@
         <v/>
       </c>
       <c r="M12">
-        <f>IF(F12="","",IF(F12&lt;5%,"&lt;5%",IF(F12&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F12="","",IF(F12&lt;5%,"&lt;5%",IF(F12&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N12" s="50">
@@ -5311,7 +5326,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="n">
+      <c r="A13" s="54" t="n">
         <v>36981</v>
       </c>
       <c r="B13" s="28" t="n">
@@ -5334,7 +5349,7 @@
         <v/>
       </c>
       <c r="G13" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C13)+0.5*COUNTIF($C$5:$C$92,C13))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C13)+(COUNTIF($C$5:$C$92,C13)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H13">
@@ -5358,7 +5373,7 @@
         <v/>
       </c>
       <c r="M13">
-        <f>IF(F13="","",IF(F13&lt;5%,"&lt;5%",IF(F13&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F13="","",IF(F13&lt;5%,"&lt;5%",IF(F13&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N13" s="50">
@@ -5383,7 +5398,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="n">
+      <c r="A14" s="54" t="n">
         <v>37072</v>
       </c>
       <c r="B14" s="28" t="n">
@@ -5406,7 +5421,7 @@
         <v/>
       </c>
       <c r="G14" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C14)+0.5*COUNTIF($C$5:$C$92,C14))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C14)+(COUNTIF($C$5:$C$92,C14)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H14">
@@ -5430,7 +5445,7 @@
         <v/>
       </c>
       <c r="M14">
-        <f>IF(F14="","",IF(F14&lt;5%,"&lt;5%",IF(F14&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F14="","",IF(F14&lt;5%,"&lt;5%",IF(F14&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N14" s="50">
@@ -5455,7 +5470,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="n">
+      <c r="A15" s="54" t="n">
         <v>37164</v>
       </c>
       <c r="B15" s="28" t="n">
@@ -5478,7 +5493,7 @@
         <v/>
       </c>
       <c r="G15" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C15)+0.5*COUNTIF($C$5:$C$92,C15))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C15)+(COUNTIF($C$5:$C$92,C15)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H15">
@@ -5502,7 +5517,7 @@
         <v/>
       </c>
       <c r="M15">
-        <f>IF(F15="","",IF(F15&lt;5%,"&lt;5%",IF(F15&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F15="","",IF(F15&lt;5%,"&lt;5%",IF(F15&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N15" s="50">
@@ -5527,7 +5542,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="n">
+      <c r="A16" s="54" t="n">
         <v>37256</v>
       </c>
       <c r="B16" s="28" t="n">
@@ -5550,7 +5565,7 @@
         <v/>
       </c>
       <c r="G16" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C16)+0.5*COUNTIF($C$5:$C$92,C16))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C16)+(COUNTIF($C$5:$C$92,C16)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H16">
@@ -5574,7 +5589,7 @@
         <v/>
       </c>
       <c r="M16">
-        <f>IF(F16="","",IF(F16&lt;5%,"&lt;5%",IF(F16&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F16="","",IF(F16&lt;5%,"&lt;5%",IF(F16&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N16" s="50">
@@ -5599,7 +5614,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="n">
+      <c r="A17" s="54" t="n">
         <v>37346</v>
       </c>
       <c r="B17" s="28" t="n">
@@ -5622,7 +5637,7 @@
         <v/>
       </c>
       <c r="G17" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C17)+0.5*COUNTIF($C$5:$C$92,C17))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C17)+(COUNTIF($C$5:$C$92,C17)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H17">
@@ -5646,7 +5661,7 @@
         <v/>
       </c>
       <c r="M17">
-        <f>IF(F17="","",IF(F17&lt;5%,"&lt;5%",IF(F17&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F17="","",IF(F17&lt;5%,"&lt;5%",IF(F17&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N17" s="50">
@@ -5671,7 +5686,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="n">
+      <c r="A18" s="54" t="n">
         <v>37437</v>
       </c>
       <c r="B18" s="28" t="n">
@@ -5694,7 +5709,7 @@
         <v/>
       </c>
       <c r="G18" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C18)+0.5*COUNTIF($C$5:$C$92,C18))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C18)+(COUNTIF($C$5:$C$92,C18)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H18">
@@ -5718,7 +5733,7 @@
         <v/>
       </c>
       <c r="M18">
-        <f>IF(F18="","",IF(F18&lt;5%,"&lt;5%",IF(F18&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F18="","",IF(F18&lt;5%,"&lt;5%",IF(F18&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N18" s="50">
@@ -5743,7 +5758,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="n">
+      <c r="A19" s="54" t="n">
         <v>37529</v>
       </c>
       <c r="B19" s="28" t="n">
@@ -5766,7 +5781,7 @@
         <v/>
       </c>
       <c r="G19" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C19)+0.5*COUNTIF($C$5:$C$92,C19))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C19)+(COUNTIF($C$5:$C$92,C19)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H19">
@@ -5790,7 +5805,7 @@
         <v/>
       </c>
       <c r="M19">
-        <f>IF(F19="","",IF(F19&lt;5%,"&lt;5%",IF(F19&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F19="","",IF(F19&lt;5%,"&lt;5%",IF(F19&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N19" s="50">
@@ -5815,7 +5830,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="n">
+      <c r="A20" s="54" t="n">
         <v>37621</v>
       </c>
       <c r="B20" s="28" t="n">
@@ -5838,7 +5853,7 @@
         <v/>
       </c>
       <c r="G20" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C20)+0.5*COUNTIF($C$5:$C$92,C20))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C20)+(COUNTIF($C$5:$C$92,C20)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H20">
@@ -5862,7 +5877,7 @@
         <v/>
       </c>
       <c r="M20">
-        <f>IF(F20="","",IF(F20&lt;5%,"&lt;5%",IF(F20&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F20="","",IF(F20&lt;5%,"&lt;5%",IF(F20&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N20" s="50">
@@ -5887,7 +5902,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="n">
+      <c r="A21" s="54" t="n">
         <v>37711</v>
       </c>
       <c r="B21" s="28" t="n">
@@ -5910,7 +5925,7 @@
         <v/>
       </c>
       <c r="G21" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C21)+0.5*COUNTIF($C$5:$C$92,C21))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C21)+(COUNTIF($C$5:$C$92,C21)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H21">
@@ -5934,7 +5949,7 @@
         <v/>
       </c>
       <c r="M21">
-        <f>IF(F21="","",IF(F21&lt;5%,"&lt;5%",IF(F21&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F21="","",IF(F21&lt;5%,"&lt;5%",IF(F21&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N21" s="50">
@@ -5959,7 +5974,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="n">
+      <c r="A22" s="54" t="n">
         <v>37802</v>
       </c>
       <c r="B22" s="28" t="n">
@@ -5982,7 +5997,7 @@
         <v/>
       </c>
       <c r="G22" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C22)+0.5*COUNTIF($C$5:$C$92,C22))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C22)+(COUNTIF($C$5:$C$92,C22)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H22">
@@ -6006,7 +6021,7 @@
         <v/>
       </c>
       <c r="M22">
-        <f>IF(F22="","",IF(F22&lt;5%,"&lt;5%",IF(F22&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F22="","",IF(F22&lt;5%,"&lt;5%",IF(F22&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N22" s="50">
@@ -6031,7 +6046,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="n">
+      <c r="A23" s="54" t="n">
         <v>37894</v>
       </c>
       <c r="B23" s="28" t="n">
@@ -6054,7 +6069,7 @@
         <v/>
       </c>
       <c r="G23" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C23)+0.5*COUNTIF($C$5:$C$92,C23))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C23)+(COUNTIF($C$5:$C$92,C23)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H23">
@@ -6078,7 +6093,7 @@
         <v/>
       </c>
       <c r="M23">
-        <f>IF(F23="","",IF(F23&lt;5%,"&lt;5%",IF(F23&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F23="","",IF(F23&lt;5%,"&lt;5%",IF(F23&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N23" s="50">
@@ -6103,7 +6118,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="n">
+      <c r="A24" s="54" t="n">
         <v>37986</v>
       </c>
       <c r="B24" s="28" t="n">
@@ -6126,7 +6141,7 @@
         <v/>
       </c>
       <c r="G24" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C24)+0.5*COUNTIF($C$5:$C$92,C24))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C24)+(COUNTIF($C$5:$C$92,C24)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H24">
@@ -6150,7 +6165,7 @@
         <v/>
       </c>
       <c r="M24">
-        <f>IF(F24="","",IF(F24&lt;5%,"&lt;5%",IF(F24&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F24="","",IF(F24&lt;5%,"&lt;5%",IF(F24&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N24" s="50">
@@ -6175,7 +6190,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="n">
+      <c r="A25" s="54" t="n">
         <v>38077</v>
       </c>
       <c r="B25" s="28" t="n">
@@ -6198,7 +6213,7 @@
         <v/>
       </c>
       <c r="G25" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C25)+0.5*COUNTIF($C$5:$C$92,C25))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C25)+(COUNTIF($C$5:$C$92,C25)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H25">
@@ -6222,7 +6237,7 @@
         <v/>
       </c>
       <c r="M25">
-        <f>IF(F25="","",IF(F25&lt;5%,"&lt;5%",IF(F25&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F25="","",IF(F25&lt;5%,"&lt;5%",IF(F25&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N25" s="50">
@@ -6247,7 +6262,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="n">
+      <c r="A26" s="54" t="n">
         <v>38168</v>
       </c>
       <c r="B26" s="28" t="n">
@@ -6270,7 +6285,7 @@
         <v/>
       </c>
       <c r="G26" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C26)+0.5*COUNTIF($C$5:$C$92,C26))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C26)+(COUNTIF($C$5:$C$92,C26)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H26">
@@ -6294,7 +6309,7 @@
         <v/>
       </c>
       <c r="M26">
-        <f>IF(F26="","",IF(F26&lt;5%,"&lt;5%",IF(F26&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F26="","",IF(F26&lt;5%,"&lt;5%",IF(F26&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N26" s="50">
@@ -6319,7 +6334,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="n">
+      <c r="A27" s="54" t="n">
         <v>38260</v>
       </c>
       <c r="B27" s="28" t="n">
@@ -6342,7 +6357,7 @@
         <v/>
       </c>
       <c r="G27" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C27)+0.5*COUNTIF($C$5:$C$92,C27))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C27)+(COUNTIF($C$5:$C$92,C27)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H27">
@@ -6366,7 +6381,7 @@
         <v/>
       </c>
       <c r="M27">
-        <f>IF(F27="","",IF(F27&lt;5%,"&lt;5%",IF(F27&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F27="","",IF(F27&lt;5%,"&lt;5%",IF(F27&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N27" s="50">
@@ -6391,7 +6406,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n">
+      <c r="A28" s="54" t="n">
         <v>38352</v>
       </c>
       <c r="B28" s="28" t="n">
@@ -6414,7 +6429,7 @@
         <v/>
       </c>
       <c r="G28" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C28)+0.5*COUNTIF($C$5:$C$92,C28))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C28)+(COUNTIF($C$5:$C$92,C28)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H28">
@@ -6438,7 +6453,7 @@
         <v/>
       </c>
       <c r="M28">
-        <f>IF(F28="","",IF(F28&lt;5%,"&lt;5%",IF(F28&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F28="","",IF(F28&lt;5%,"&lt;5%",IF(F28&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N28" s="50">
@@ -6463,7 +6478,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="n">
+      <c r="A29" s="54" t="n">
         <v>38442</v>
       </c>
       <c r="B29" s="28" t="n">
@@ -6486,7 +6501,7 @@
         <v/>
       </c>
       <c r="G29" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C29)+0.5*COUNTIF($C$5:$C$92,C29))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C29)+(COUNTIF($C$5:$C$92,C29)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H29">
@@ -6510,7 +6525,7 @@
         <v/>
       </c>
       <c r="M29">
-        <f>IF(F29="","",IF(F29&lt;5%,"&lt;5%",IF(F29&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F29="","",IF(F29&lt;5%,"&lt;5%",IF(F29&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N29" s="50">
@@ -6535,7 +6550,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="n">
+      <c r="A30" s="54" t="n">
         <v>38533</v>
       </c>
       <c r="B30" s="28" t="n">
@@ -6558,7 +6573,7 @@
         <v/>
       </c>
       <c r="G30" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C30)+0.5*COUNTIF($C$5:$C$92,C30))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C30)+(COUNTIF($C$5:$C$92,C30)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H30">
@@ -6582,7 +6597,7 @@
         <v/>
       </c>
       <c r="M30">
-        <f>IF(F30="","",IF(F30&lt;5%,"&lt;5%",IF(F30&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F30="","",IF(F30&lt;5%,"&lt;5%",IF(F30&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N30" s="50">
@@ -6607,7 +6622,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="n">
+      <c r="A31" s="54" t="n">
         <v>38625</v>
       </c>
       <c r="B31" s="28" t="n">
@@ -6630,7 +6645,7 @@
         <v/>
       </c>
       <c r="G31" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C31)+0.5*COUNTIF($C$5:$C$92,C31))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C31)+(COUNTIF($C$5:$C$92,C31)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H31">
@@ -6654,7 +6669,7 @@
         <v/>
       </c>
       <c r="M31">
-        <f>IF(F31="","",IF(F31&lt;5%,"&lt;5%",IF(F31&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F31="","",IF(F31&lt;5%,"&lt;5%",IF(F31&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N31" s="50">
@@ -6679,7 +6694,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="n">
+      <c r="A32" s="54" t="n">
         <v>38717</v>
       </c>
       <c r="B32" s="28" t="n">
@@ -6702,7 +6717,7 @@
         <v/>
       </c>
       <c r="G32" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C32)+0.5*COUNTIF($C$5:$C$92,C32))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C32)+(COUNTIF($C$5:$C$92,C32)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H32">
@@ -6726,7 +6741,7 @@
         <v/>
       </c>
       <c r="M32">
-        <f>IF(F32="","",IF(F32&lt;5%,"&lt;5%",IF(F32&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F32="","",IF(F32&lt;5%,"&lt;5%",IF(F32&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N32" s="50">
@@ -6751,7 +6766,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="n">
+      <c r="A33" s="54" t="n">
         <v>38807</v>
       </c>
       <c r="B33" s="28" t="n">
@@ -6774,7 +6789,7 @@
         <v/>
       </c>
       <c r="G33" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C33)+0.5*COUNTIF($C$5:$C$92,C33))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C33)+(COUNTIF($C$5:$C$92,C33)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H33">
@@ -6798,7 +6813,7 @@
         <v/>
       </c>
       <c r="M33">
-        <f>IF(F33="","",IF(F33&lt;5%,"&lt;5%",IF(F33&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F33="","",IF(F33&lt;5%,"&lt;5%",IF(F33&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N33" s="50">
@@ -6823,7 +6838,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="n">
+      <c r="A34" s="54" t="n">
         <v>38898</v>
       </c>
       <c r="B34" s="28" t="n">
@@ -6846,7 +6861,7 @@
         <v/>
       </c>
       <c r="G34" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C34)+0.5*COUNTIF($C$5:$C$92,C34))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C34)+(COUNTIF($C$5:$C$92,C34)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H34">
@@ -6870,7 +6885,7 @@
         <v/>
       </c>
       <c r="M34">
-        <f>IF(F34="","",IF(F34&lt;5%,"&lt;5%",IF(F34&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F34="","",IF(F34&lt;5%,"&lt;5%",IF(F34&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N34" s="50">
@@ -6895,7 +6910,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="n">
+      <c r="A35" s="54" t="n">
         <v>38990</v>
       </c>
       <c r="B35" s="28" t="n">
@@ -6918,7 +6933,7 @@
         <v/>
       </c>
       <c r="G35" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C35)+0.5*COUNTIF($C$5:$C$92,C35))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C35)+(COUNTIF($C$5:$C$92,C35)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H35">
@@ -6942,7 +6957,7 @@
         <v/>
       </c>
       <c r="M35">
-        <f>IF(F35="","",IF(F35&lt;5%,"&lt;5%",IF(F35&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F35="","",IF(F35&lt;5%,"&lt;5%",IF(F35&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N35" s="50">
@@ -6967,7 +6982,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="n">
+      <c r="A36" s="54" t="n">
         <v>39082</v>
       </c>
       <c r="B36" s="28" t="n">
@@ -6990,7 +7005,7 @@
         <v/>
       </c>
       <c r="G36" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C36)+0.5*COUNTIF($C$5:$C$92,C36))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C36)+(COUNTIF($C$5:$C$92,C36)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H36">
@@ -7014,7 +7029,7 @@
         <v/>
       </c>
       <c r="M36">
-        <f>IF(F36="","",IF(F36&lt;5%,"&lt;5%",IF(F36&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F36="","",IF(F36&lt;5%,"&lt;5%",IF(F36&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N36" s="50">
@@ -7039,7 +7054,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="n">
+      <c r="A37" s="54" t="n">
         <v>39172</v>
       </c>
       <c r="B37" s="28" t="n">
@@ -7062,7 +7077,7 @@
         <v/>
       </c>
       <c r="G37" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C37)+0.5*COUNTIF($C$5:$C$92,C37))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C37)+(COUNTIF($C$5:$C$92,C37)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H37">
@@ -7086,7 +7101,7 @@
         <v/>
       </c>
       <c r="M37">
-        <f>IF(F37="","",IF(F37&lt;5%,"&lt;5%",IF(F37&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F37="","",IF(F37&lt;5%,"&lt;5%",IF(F37&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N37" s="50">
@@ -7111,7 +7126,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="n">
+      <c r="A38" s="54" t="n">
         <v>39263</v>
       </c>
       <c r="B38" s="28" t="n">
@@ -7134,7 +7149,7 @@
         <v/>
       </c>
       <c r="G38" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C38)+0.5*COUNTIF($C$5:$C$92,C38))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C38)+(COUNTIF($C$5:$C$92,C38)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H38">
@@ -7158,7 +7173,7 @@
         <v/>
       </c>
       <c r="M38">
-        <f>IF(F38="","",IF(F38&lt;5%,"&lt;5%",IF(F38&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F38="","",IF(F38&lt;5%,"&lt;5%",IF(F38&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N38" s="50">
@@ -7183,7 +7198,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="n">
+      <c r="A39" s="54" t="n">
         <v>39355</v>
       </c>
       <c r="B39" s="28" t="n">
@@ -7206,7 +7221,7 @@
         <v/>
       </c>
       <c r="G39" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C39)+0.5*COUNTIF($C$5:$C$92,C39))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C39)+(COUNTIF($C$5:$C$92,C39)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H39">
@@ -7230,7 +7245,7 @@
         <v/>
       </c>
       <c r="M39">
-        <f>IF(F39="","",IF(F39&lt;5%,"&lt;5%",IF(F39&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F39="","",IF(F39&lt;5%,"&lt;5%",IF(F39&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N39" s="50">
@@ -7255,7 +7270,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="n">
+      <c r="A40" s="54" t="n">
         <v>39447</v>
       </c>
       <c r="B40" s="28" t="n">
@@ -7278,7 +7293,7 @@
         <v/>
       </c>
       <c r="G40" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C40)+0.5*COUNTIF($C$5:$C$92,C40))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C40)+(COUNTIF($C$5:$C$92,C40)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H40">
@@ -7302,7 +7317,7 @@
         <v/>
       </c>
       <c r="M40">
-        <f>IF(F40="","",IF(F40&lt;5%,"&lt;5%",IF(F40&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F40="","",IF(F40&lt;5%,"&lt;5%",IF(F40&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N40" s="50">
@@ -7327,7 +7342,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="n">
+      <c r="A41" s="54" t="n">
         <v>39538</v>
       </c>
       <c r="B41" s="28" t="n">
@@ -7350,7 +7365,7 @@
         <v/>
       </c>
       <c r="G41" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C41)+0.5*COUNTIF($C$5:$C$92,C41))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C41)+(COUNTIF($C$5:$C$92,C41)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H41">
@@ -7374,7 +7389,7 @@
         <v/>
       </c>
       <c r="M41">
-        <f>IF(F41="","",IF(F41&lt;5%,"&lt;5%",IF(F41&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F41="","",IF(F41&lt;5%,"&lt;5%",IF(F41&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N41" s="50">
@@ -7399,7 +7414,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="n">
+      <c r="A42" s="54" t="n">
         <v>39629</v>
       </c>
       <c r="B42" s="28" t="n">
@@ -7422,7 +7437,7 @@
         <v/>
       </c>
       <c r="G42" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C42)+0.5*COUNTIF($C$5:$C$92,C42))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C42)+(COUNTIF($C$5:$C$92,C42)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H42">
@@ -7446,7 +7461,7 @@
         <v/>
       </c>
       <c r="M42">
-        <f>IF(F42="","",IF(F42&lt;5%,"&lt;5%",IF(F42&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F42="","",IF(F42&lt;5%,"&lt;5%",IF(F42&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N42" s="50">
@@ -7471,7 +7486,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="n">
+      <c r="A43" s="54" t="n">
         <v>39721</v>
       </c>
       <c r="B43" s="28" t="n">
@@ -7494,7 +7509,7 @@
         <v/>
       </c>
       <c r="G43" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C43)+0.5*COUNTIF($C$5:$C$92,C43))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C43)+(COUNTIF($C$5:$C$92,C43)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H43">
@@ -7518,7 +7533,7 @@
         <v/>
       </c>
       <c r="M43">
-        <f>IF(F43="","",IF(F43&lt;5%,"&lt;5%",IF(F43&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F43="","",IF(F43&lt;5%,"&lt;5%",IF(F43&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N43" s="50">
@@ -7543,7 +7558,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="27" t="n">
+      <c r="A44" s="54" t="n">
         <v>39813</v>
       </c>
       <c r="B44" s="28" t="n">
@@ -7566,7 +7581,7 @@
         <v/>
       </c>
       <c r="G44" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C44)+0.5*COUNTIF($C$5:$C$92,C44))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C44)+(COUNTIF($C$5:$C$92,C44)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H44">
@@ -7590,7 +7605,7 @@
         <v/>
       </c>
       <c r="M44">
-        <f>IF(F44="","",IF(F44&lt;5%,"&lt;5%",IF(F44&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F44="","",IF(F44&lt;5%,"&lt;5%",IF(F44&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N44" s="50">
@@ -7615,7 +7630,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="n">
+      <c r="A45" s="54" t="n">
         <v>39903</v>
       </c>
       <c r="B45" s="28" t="n">
@@ -7638,7 +7653,7 @@
         <v/>
       </c>
       <c r="G45" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C45)+0.5*COUNTIF($C$5:$C$92,C45))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C45)+(COUNTIF($C$5:$C$92,C45)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H45">
@@ -7662,7 +7677,7 @@
         <v/>
       </c>
       <c r="M45">
-        <f>IF(F45="","",IF(F45&lt;5%,"&lt;5%",IF(F45&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F45="","",IF(F45&lt;5%,"&lt;5%",IF(F45&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N45" s="50">
@@ -7687,7 +7702,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="27" t="n">
+      <c r="A46" s="54" t="n">
         <v>39994</v>
       </c>
       <c r="B46" s="28" t="n">
@@ -7710,7 +7725,7 @@
         <v/>
       </c>
       <c r="G46" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C46)+0.5*COUNTIF($C$5:$C$92,C46))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C46)+(COUNTIF($C$5:$C$92,C46)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H46">
@@ -7734,7 +7749,7 @@
         <v/>
       </c>
       <c r="M46">
-        <f>IF(F46="","",IF(F46&lt;5%,"&lt;5%",IF(F46&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F46="","",IF(F46&lt;5%,"&lt;5%",IF(F46&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N46" s="50">
@@ -7759,7 +7774,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="27" t="n">
+      <c r="A47" s="54" t="n">
         <v>40086</v>
       </c>
       <c r="B47" s="28" t="n">
@@ -7782,7 +7797,7 @@
         <v/>
       </c>
       <c r="G47" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C47)+0.5*COUNTIF($C$5:$C$92,C47))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C47)+(COUNTIF($C$5:$C$92,C47)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H47">
@@ -7806,7 +7821,7 @@
         <v/>
       </c>
       <c r="M47">
-        <f>IF(F47="","",IF(F47&lt;5%,"&lt;5%",IF(F47&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F47="","",IF(F47&lt;5%,"&lt;5%",IF(F47&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N47" s="50">
@@ -7831,7 +7846,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="27" t="n">
+      <c r="A48" s="54" t="n">
         <v>40178</v>
       </c>
       <c r="B48" s="28" t="n">
@@ -7854,7 +7869,7 @@
         <v/>
       </c>
       <c r="G48" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C48)+0.5*COUNTIF($C$5:$C$92,C48))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C48)+(COUNTIF($C$5:$C$92,C48)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H48">
@@ -7878,7 +7893,7 @@
         <v/>
       </c>
       <c r="M48">
-        <f>IF(F48="","",IF(F48&lt;5%,"&lt;5%",IF(F48&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F48="","",IF(F48&lt;5%,"&lt;5%",IF(F48&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N48" s="50">
@@ -7903,7 +7918,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="27" t="n">
+      <c r="A49" s="54" t="n">
         <v>40268</v>
       </c>
       <c r="B49" s="28" t="n">
@@ -7926,7 +7941,7 @@
         <v/>
       </c>
       <c r="G49" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C49)+0.5*COUNTIF($C$5:$C$92,C49))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C49)+(COUNTIF($C$5:$C$92,C49)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H49">
@@ -7950,7 +7965,7 @@
         <v/>
       </c>
       <c r="M49">
-        <f>IF(F49="","",IF(F49&lt;5%,"&lt;5%",IF(F49&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F49="","",IF(F49&lt;5%,"&lt;5%",IF(F49&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N49" s="50">
@@ -7975,7 +7990,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="n">
+      <c r="A50" s="54" t="n">
         <v>40359</v>
       </c>
       <c r="B50" s="28" t="n">
@@ -7998,7 +8013,7 @@
         <v/>
       </c>
       <c r="G50" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C50)+0.5*COUNTIF($C$5:$C$92,C50))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C50)+(COUNTIF($C$5:$C$92,C50)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H50">
@@ -8022,7 +8037,7 @@
         <v/>
       </c>
       <c r="M50">
-        <f>IF(F50="","",IF(F50&lt;5%,"&lt;5%",IF(F50&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F50="","",IF(F50&lt;5%,"&lt;5%",IF(F50&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N50" s="50">
@@ -8047,7 +8062,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="27" t="n">
+      <c r="A51" s="54" t="n">
         <v>40451</v>
       </c>
       <c r="B51" s="28" t="n">
@@ -8070,7 +8085,7 @@
         <v/>
       </c>
       <c r="G51" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C51)+0.5*COUNTIF($C$5:$C$92,C51))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C51)+(COUNTIF($C$5:$C$92,C51)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H51">
@@ -8094,7 +8109,7 @@
         <v/>
       </c>
       <c r="M51">
-        <f>IF(F51="","",IF(F51&lt;5%,"&lt;5%",IF(F51&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F51="","",IF(F51&lt;5%,"&lt;5%",IF(F51&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N51" s="50">
@@ -8119,7 +8134,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="27" t="n">
+      <c r="A52" s="54" t="n">
         <v>40543</v>
       </c>
       <c r="B52" s="28" t="n">
@@ -8142,7 +8157,7 @@
         <v/>
       </c>
       <c r="G52" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C52)+0.5*COUNTIF($C$5:$C$92,C52))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C52)+(COUNTIF($C$5:$C$92,C52)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H52">
@@ -8166,7 +8181,7 @@
         <v/>
       </c>
       <c r="M52">
-        <f>IF(F52="","",IF(F52&lt;5%,"&lt;5%",IF(F52&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F52="","",IF(F52&lt;5%,"&lt;5%",IF(F52&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N52" s="50">
@@ -8191,7 +8206,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="27" t="n">
+      <c r="A53" s="54" t="n">
         <v>40633</v>
       </c>
       <c r="B53" s="28" t="n">
@@ -8214,7 +8229,7 @@
         <v/>
       </c>
       <c r="G53" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C53)+0.5*COUNTIF($C$5:$C$92,C53))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C53)+(COUNTIF($C$5:$C$92,C53)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H53">
@@ -8238,7 +8253,7 @@
         <v/>
       </c>
       <c r="M53">
-        <f>IF(F53="","",IF(F53&lt;5%,"&lt;5%",IF(F53&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F53="","",IF(F53&lt;5%,"&lt;5%",IF(F53&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N53" s="50">
@@ -8263,7 +8278,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="27" t="n">
+      <c r="A54" s="54" t="n">
         <v>40724</v>
       </c>
       <c r="B54" s="28" t="n">
@@ -8286,7 +8301,7 @@
         <v/>
       </c>
       <c r="G54" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C54)+0.5*COUNTIF($C$5:$C$92,C54))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C54)+(COUNTIF($C$5:$C$92,C54)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H54">
@@ -8310,7 +8325,7 @@
         <v/>
       </c>
       <c r="M54">
-        <f>IF(F54="","",IF(F54&lt;5%,"&lt;5%",IF(F54&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F54="","",IF(F54&lt;5%,"&lt;5%",IF(F54&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N54" s="50">
@@ -8335,7 +8350,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="27" t="n">
+      <c r="A55" s="54" t="n">
         <v>40816</v>
       </c>
       <c r="B55" s="28" t="n">
@@ -8358,7 +8373,7 @@
         <v/>
       </c>
       <c r="G55" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C55)+0.5*COUNTIF($C$5:$C$92,C55))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C55)+(COUNTIF($C$5:$C$92,C55)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H55">
@@ -8382,7 +8397,7 @@
         <v/>
       </c>
       <c r="M55">
-        <f>IF(F55="","",IF(F55&lt;5%,"&lt;5%",IF(F55&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F55="","",IF(F55&lt;5%,"&lt;5%",IF(F55&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N55" s="50">
@@ -8407,7 +8422,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="27" t="n">
+      <c r="A56" s="54" t="n">
         <v>40908</v>
       </c>
       <c r="B56" s="28" t="n">
@@ -8430,7 +8445,7 @@
         <v/>
       </c>
       <c r="G56" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C56)+0.5*COUNTIF($C$5:$C$92,C56))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C56)+(COUNTIF($C$5:$C$92,C56)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H56">
@@ -8454,7 +8469,7 @@
         <v/>
       </c>
       <c r="M56">
-        <f>IF(F56="","",IF(F56&lt;5%,"&lt;5%",IF(F56&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F56="","",IF(F56&lt;5%,"&lt;5%",IF(F56&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N56" s="50">
@@ -8479,7 +8494,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="27" t="n">
+      <c r="A57" s="54" t="n">
         <v>40999</v>
       </c>
       <c r="B57" s="28" t="n">
@@ -8502,7 +8517,7 @@
         <v/>
       </c>
       <c r="G57" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C57)+0.5*COUNTIF($C$5:$C$92,C57))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C57)+(COUNTIF($C$5:$C$92,C57)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H57">
@@ -8526,7 +8541,7 @@
         <v/>
       </c>
       <c r="M57">
-        <f>IF(F57="","",IF(F57&lt;5%,"&lt;5%",IF(F57&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F57="","",IF(F57&lt;5%,"&lt;5%",IF(F57&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N57" s="50">
@@ -8551,7 +8566,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="n">
+      <c r="A58" s="54" t="n">
         <v>41090</v>
       </c>
       <c r="B58" s="28" t="n">
@@ -8574,7 +8589,7 @@
         <v/>
       </c>
       <c r="G58" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C58)+0.5*COUNTIF($C$5:$C$92,C58))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C58)+(COUNTIF($C$5:$C$92,C58)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H58">
@@ -8598,7 +8613,7 @@
         <v/>
       </c>
       <c r="M58">
-        <f>IF(F58="","",IF(F58&lt;5%,"&lt;5%",IF(F58&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F58="","",IF(F58&lt;5%,"&lt;5%",IF(F58&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N58" s="50">
@@ -8623,7 +8638,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="27" t="n">
+      <c r="A59" s="54" t="n">
         <v>41182</v>
       </c>
       <c r="B59" s="28" t="n">
@@ -8646,7 +8661,7 @@
         <v/>
       </c>
       <c r="G59" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C59)+0.5*COUNTIF($C$5:$C$92,C59))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C59)+(COUNTIF($C$5:$C$92,C59)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H59">
@@ -8670,7 +8685,7 @@
         <v/>
       </c>
       <c r="M59">
-        <f>IF(F59="","",IF(F59&lt;5%,"&lt;5%",IF(F59&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F59="","",IF(F59&lt;5%,"&lt;5%",IF(F59&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N59" s="50">
@@ -8695,7 +8710,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="27" t="n">
+      <c r="A60" s="54" t="n">
         <v>41274</v>
       </c>
       <c r="B60" s="28" t="n">
@@ -8718,7 +8733,7 @@
         <v/>
       </c>
       <c r="G60" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C60)+0.5*COUNTIF($C$5:$C$92,C60))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C60)+(COUNTIF($C$5:$C$92,C60)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H60">
@@ -8742,7 +8757,7 @@
         <v/>
       </c>
       <c r="M60">
-        <f>IF(F60="","",IF(F60&lt;5%,"&lt;5%",IF(F60&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F60="","",IF(F60&lt;5%,"&lt;5%",IF(F60&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N60" s="50">
@@ -8767,7 +8782,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="27" t="n">
+      <c r="A61" s="54" t="n">
         <v>41364</v>
       </c>
       <c r="B61" s="28" t="n">
@@ -8790,7 +8805,7 @@
         <v/>
       </c>
       <c r="G61" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C61)+0.5*COUNTIF($C$5:$C$92,C61))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C61)+(COUNTIF($C$5:$C$92,C61)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H61">
@@ -8814,7 +8829,7 @@
         <v/>
       </c>
       <c r="M61">
-        <f>IF(F61="","",IF(F61&lt;5%,"&lt;5%",IF(F61&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F61="","",IF(F61&lt;5%,"&lt;5%",IF(F61&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N61" s="50">
@@ -8839,7 +8854,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="27" t="n">
+      <c r="A62" s="54" t="n">
         <v>41455</v>
       </c>
       <c r="B62" s="28" t="n">
@@ -8862,7 +8877,7 @@
         <v/>
       </c>
       <c r="G62" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C62)+0.5*COUNTIF($C$5:$C$92,C62))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C62)+(COUNTIF($C$5:$C$92,C62)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H62">
@@ -8886,7 +8901,7 @@
         <v/>
       </c>
       <c r="M62">
-        <f>IF(F62="","",IF(F62&lt;5%,"&lt;5%",IF(F62&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F62="","",IF(F62&lt;5%,"&lt;5%",IF(F62&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N62" s="50">
@@ -8911,7 +8926,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="27" t="n">
+      <c r="A63" s="54" t="n">
         <v>41547</v>
       </c>
       <c r="B63" s="28" t="n">
@@ -8934,7 +8949,7 @@
         <v/>
       </c>
       <c r="G63" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C63)+0.5*COUNTIF($C$5:$C$92,C63))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C63)+(COUNTIF($C$5:$C$92,C63)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H63">
@@ -8958,7 +8973,7 @@
         <v/>
       </c>
       <c r="M63">
-        <f>IF(F63="","",IF(F63&lt;5%,"&lt;5%",IF(F63&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F63="","",IF(F63&lt;5%,"&lt;5%",IF(F63&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N63" s="50">
@@ -8983,7 +8998,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="27" t="n">
+      <c r="A64" s="54" t="n">
         <v>41639</v>
       </c>
       <c r="B64" s="28" t="n">
@@ -9006,7 +9021,7 @@
         <v/>
       </c>
       <c r="G64" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C64)+0.5*COUNTIF($C$5:$C$92,C64))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C64)+(COUNTIF($C$5:$C$92,C64)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H64">
@@ -9030,7 +9045,7 @@
         <v/>
       </c>
       <c r="M64">
-        <f>IF(F64="","",IF(F64&lt;5%,"&lt;5%",IF(F64&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F64="","",IF(F64&lt;5%,"&lt;5%",IF(F64&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N64" s="50">
@@ -9055,7 +9070,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="27" t="n">
+      <c r="A65" s="54" t="n">
         <v>41729</v>
       </c>
       <c r="B65" s="28" t="n">
@@ -9078,7 +9093,7 @@
         <v/>
       </c>
       <c r="G65" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C65)+0.5*COUNTIF($C$5:$C$92,C65))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C65)+(COUNTIF($C$5:$C$92,C65)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H65">
@@ -9102,7 +9117,7 @@
         <v/>
       </c>
       <c r="M65">
-        <f>IF(F65="","",IF(F65&lt;5%,"&lt;5%",IF(F65&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F65="","",IF(F65&lt;5%,"&lt;5%",IF(F65&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N65" s="50">
@@ -9127,7 +9142,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="n">
+      <c r="A66" s="54" t="n">
         <v>41820</v>
       </c>
       <c r="B66" s="28" t="n">
@@ -9150,7 +9165,7 @@
         <v/>
       </c>
       <c r="G66" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C66)+0.5*COUNTIF($C$5:$C$92,C66))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C66)+(COUNTIF($C$5:$C$92,C66)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H66">
@@ -9174,7 +9189,7 @@
         <v/>
       </c>
       <c r="M66">
-        <f>IF(F66="","",IF(F66&lt;5%,"&lt;5%",IF(F66&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F66="","",IF(F66&lt;5%,"&lt;5%",IF(F66&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N66" s="50">
@@ -9199,7 +9214,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="27" t="n">
+      <c r="A67" s="54" t="n">
         <v>41912</v>
       </c>
       <c r="B67" s="28" t="n">
@@ -9222,7 +9237,7 @@
         <v/>
       </c>
       <c r="G67" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C67)+0.5*COUNTIF($C$5:$C$92,C67))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C67)+(COUNTIF($C$5:$C$92,C67)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H67">
@@ -9246,7 +9261,7 @@
         <v/>
       </c>
       <c r="M67">
-        <f>IF(F67="","",IF(F67&lt;5%,"&lt;5%",IF(F67&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F67="","",IF(F67&lt;5%,"&lt;5%",IF(F67&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N67" s="50">
@@ -9271,7 +9286,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="27" t="n">
+      <c r="A68" s="54" t="n">
         <v>42004</v>
       </c>
       <c r="B68" s="28" t="n">
@@ -9294,7 +9309,7 @@
         <v/>
       </c>
       <c r="G68" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C68)+0.5*COUNTIF($C$5:$C$92,C68))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C68)+(COUNTIF($C$5:$C$92,C68)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H68">
@@ -9318,7 +9333,7 @@
         <v/>
       </c>
       <c r="M68">
-        <f>IF(F68="","",IF(F68&lt;5%,"&lt;5%",IF(F68&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F68="","",IF(F68&lt;5%,"&lt;5%",IF(F68&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N68" s="50">
@@ -9343,7 +9358,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="27" t="n">
+      <c r="A69" s="54" t="n">
         <v>42094</v>
       </c>
       <c r="B69" s="28" t="n">
@@ -9366,7 +9381,7 @@
         <v/>
       </c>
       <c r="G69" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C69)+0.5*COUNTIF($C$5:$C$92,C69))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C69)+(COUNTIF($C$5:$C$92,C69)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H69">
@@ -9390,7 +9405,7 @@
         <v/>
       </c>
       <c r="M69">
-        <f>IF(F69="","",IF(F69&lt;5%,"&lt;5%",IF(F69&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F69="","",IF(F69&lt;5%,"&lt;5%",IF(F69&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N69" s="50">
@@ -9415,7 +9430,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="27" t="n">
+      <c r="A70" s="54" t="n">
         <v>42185</v>
       </c>
       <c r="B70" s="28" t="n">
@@ -9438,7 +9453,7 @@
         <v/>
       </c>
       <c r="G70" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C70)+0.5*COUNTIF($C$5:$C$92,C70))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C70)+(COUNTIF($C$5:$C$92,C70)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H70">
@@ -9462,7 +9477,7 @@
         <v/>
       </c>
       <c r="M70">
-        <f>IF(F70="","",IF(F70&lt;5%,"&lt;5%",IF(F70&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F70="","",IF(F70&lt;5%,"&lt;5%",IF(F70&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N70" s="50">
@@ -9487,7 +9502,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="27" t="n">
+      <c r="A71" s="54" t="n">
         <v>42277</v>
       </c>
       <c r="B71" s="28" t="n">
@@ -9510,7 +9525,7 @@
         <v/>
       </c>
       <c r="G71" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C71)+0.5*COUNTIF($C$5:$C$92,C71))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C71)+(COUNTIF($C$5:$C$92,C71)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H71">
@@ -9534,7 +9549,7 @@
         <v/>
       </c>
       <c r="M71">
-        <f>IF(F71="","",IF(F71&lt;5%,"&lt;5%",IF(F71&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F71="","",IF(F71&lt;5%,"&lt;5%",IF(F71&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N71" s="50">
@@ -9559,7 +9574,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="27" t="n">
+      <c r="A72" s="54" t="n">
         <v>42369</v>
       </c>
       <c r="B72" s="28" t="n">
@@ -9582,7 +9597,7 @@
         <v/>
       </c>
       <c r="G72" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C72)+0.5*COUNTIF($C$5:$C$92,C72))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C72)+(COUNTIF($C$5:$C$92,C72)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H72">
@@ -9606,7 +9621,7 @@
         <v/>
       </c>
       <c r="M72">
-        <f>IF(F72="","",IF(F72&lt;5%,"&lt;5%",IF(F72&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F72="","",IF(F72&lt;5%,"&lt;5%",IF(F72&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N72" s="50">
@@ -9631,7 +9646,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="27" t="n">
+      <c r="A73" s="54" t="n">
         <v>42460</v>
       </c>
       <c r="B73" s="28" t="n">
@@ -9654,7 +9669,7 @@
         <v/>
       </c>
       <c r="G73" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C73)+0.5*COUNTIF($C$5:$C$92,C73))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C73)+(COUNTIF($C$5:$C$92,C73)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H73">
@@ -9678,7 +9693,7 @@
         <v/>
       </c>
       <c r="M73">
-        <f>IF(F73="","",IF(F73&lt;5%,"&lt;5%",IF(F73&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F73="","",IF(F73&lt;5%,"&lt;5%",IF(F73&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N73" s="50">
@@ -9703,7 +9718,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="27" t="n">
+      <c r="A74" s="54" t="n">
         <v>42551</v>
       </c>
       <c r="B74" s="28" t="n">
@@ -9726,7 +9741,7 @@
         <v/>
       </c>
       <c r="G74" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C74)+0.5*COUNTIF($C$5:$C$92,C74))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C74)+(COUNTIF($C$5:$C$92,C74)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H74">
@@ -9750,7 +9765,7 @@
         <v/>
       </c>
       <c r="M74">
-        <f>IF(F74="","",IF(F74&lt;5%,"&lt;5%",IF(F74&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F74="","",IF(F74&lt;5%,"&lt;5%",IF(F74&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N74" s="50">
@@ -9775,7 +9790,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="27" t="n">
+      <c r="A75" s="54" t="n">
         <v>42643</v>
       </c>
       <c r="B75" s="28" t="n">
@@ -9798,7 +9813,7 @@
         <v/>
       </c>
       <c r="G75" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C75)+0.5*COUNTIF($C$5:$C$92,C75))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C75)+(COUNTIF($C$5:$C$92,C75)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H75">
@@ -9819,7 +9834,7 @@
       </c>
       <c r="L75" s="50" t="inlineStr"/>
       <c r="M75">
-        <f>IF(F75="","",IF(F75&lt;5%,"&lt;5%",IF(F75&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F75="","",IF(F75&lt;5%,"&lt;5%",IF(F75&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N75" s="50">
@@ -9844,7 +9859,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="27" t="n">
+      <c r="A76" s="54" t="n">
         <v>42735</v>
       </c>
       <c r="B76" s="28" t="n">
@@ -9867,7 +9882,7 @@
         <v/>
       </c>
       <c r="G76" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C76)+0.5*COUNTIF($C$5:$C$92,C76))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C76)+(COUNTIF($C$5:$C$92,C76)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H76">
@@ -9888,7 +9903,7 @@
       </c>
       <c r="L76" s="50" t="inlineStr"/>
       <c r="M76">
-        <f>IF(F76="","",IF(F76&lt;5%,"&lt;5%",IF(F76&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F76="","",IF(F76&lt;5%,"&lt;5%",IF(F76&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N76" s="50">
@@ -9913,7 +9928,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="27" t="n">
+      <c r="A77" s="54" t="n">
         <v>42825</v>
       </c>
       <c r="B77" s="28" t="n">
@@ -9936,7 +9951,7 @@
         <v/>
       </c>
       <c r="G77" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C77)+0.5*COUNTIF($C$5:$C$92,C77))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C77)+(COUNTIF($C$5:$C$92,C77)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H77">
@@ -9957,7 +9972,7 @@
       </c>
       <c r="L77" s="50" t="inlineStr"/>
       <c r="M77">
-        <f>IF(F77="","",IF(F77&lt;5%,"&lt;5%",IF(F77&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F77="","",IF(F77&lt;5%,"&lt;5%",IF(F77&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N77" s="50">
@@ -9982,7 +9997,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="27" t="n">
+      <c r="A78" s="54" t="n">
         <v>42916</v>
       </c>
       <c r="B78" s="28" t="n">
@@ -10005,7 +10020,7 @@
         <v/>
       </c>
       <c r="G78" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C78)+0.5*COUNTIF($C$5:$C$92,C78))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C78)+(COUNTIF($C$5:$C$92,C78)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H78">
@@ -10026,7 +10041,7 @@
       </c>
       <c r="L78" s="50" t="inlineStr"/>
       <c r="M78">
-        <f>IF(F78="","",IF(F78&lt;5%,"&lt;5%",IF(F78&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F78="","",IF(F78&lt;5%,"&lt;5%",IF(F78&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N78" s="50">
@@ -10051,7 +10066,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="27" t="n">
+      <c r="A79" s="54" t="n">
         <v>43008</v>
       </c>
       <c r="B79" s="28" t="n">
@@ -10074,7 +10089,7 @@
         <v/>
       </c>
       <c r="G79" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C79)+0.5*COUNTIF($C$5:$C$92,C79))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C79)+(COUNTIF($C$5:$C$92,C79)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H79">
@@ -10095,7 +10110,7 @@
       </c>
       <c r="L79" s="50" t="inlineStr"/>
       <c r="M79">
-        <f>IF(F79="","",IF(F79&lt;5%,"&lt;5%",IF(F79&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F79="","",IF(F79&lt;5%,"&lt;5%",IF(F79&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N79" s="50">
@@ -10120,7 +10135,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="27" t="n">
+      <c r="A80" s="54" t="n">
         <v>43100</v>
       </c>
       <c r="B80" s="28" t="n">
@@ -10143,7 +10158,7 @@
         <v/>
       </c>
       <c r="G80" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C80)+0.5*COUNTIF($C$5:$C$92,C80))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C80)+(COUNTIF($C$5:$C$92,C80)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H80">
@@ -10164,7 +10179,7 @@
       </c>
       <c r="L80" s="50" t="inlineStr"/>
       <c r="M80">
-        <f>IF(F80="","",IF(F80&lt;5%,"&lt;5%",IF(F80&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F80="","",IF(F80&lt;5%,"&lt;5%",IF(F80&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N80" s="50">
@@ -10189,7 +10204,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="27" t="n">
+      <c r="A81" s="54" t="n">
         <v>43190</v>
       </c>
       <c r="B81" s="28" t="n">
@@ -10212,7 +10227,7 @@
         <v/>
       </c>
       <c r="G81" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C81)+0.5*COUNTIF($C$5:$C$92,C81))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C81)+(COUNTIF($C$5:$C$92,C81)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H81">
@@ -10233,7 +10248,7 @@
       </c>
       <c r="L81" s="50" t="inlineStr"/>
       <c r="M81">
-        <f>IF(F81="","",IF(F81&lt;5%,"&lt;5%",IF(F81&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F81="","",IF(F81&lt;5%,"&lt;5%",IF(F81&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N81" s="50">
@@ -10258,7 +10273,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="27" t="n">
+      <c r="A82" s="54" t="n">
         <v>43281</v>
       </c>
       <c r="B82" s="28" t="n">
@@ -10281,7 +10296,7 @@
         <v/>
       </c>
       <c r="G82" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C82)+0.5*COUNTIF($C$5:$C$92,C82))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C82)+(COUNTIF($C$5:$C$92,C82)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H82">
@@ -10302,7 +10317,7 @@
       </c>
       <c r="L82" s="50" t="inlineStr"/>
       <c r="M82">
-        <f>IF(F82="","",IF(F82&lt;5%,"&lt;5%",IF(F82&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F82="","",IF(F82&lt;5%,"&lt;5%",IF(F82&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N82" s="50">
@@ -10327,7 +10342,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="27" t="n">
+      <c r="A83" s="54" t="n">
         <v>43373</v>
       </c>
       <c r="B83" s="28" t="n">
@@ -10350,7 +10365,7 @@
         <v/>
       </c>
       <c r="G83" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C83)+0.5*COUNTIF($C$5:$C$92,C83))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C83)+(COUNTIF($C$5:$C$92,C83)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H83">
@@ -10371,7 +10386,7 @@
       </c>
       <c r="L83" s="50" t="inlineStr"/>
       <c r="M83">
-        <f>IF(F83="","",IF(F83&lt;5%,"&lt;5%",IF(F83&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F83="","",IF(F83&lt;5%,"&lt;5%",IF(F83&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N83" s="50">
@@ -10396,7 +10411,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="27" t="n">
+      <c r="A84" s="54" t="n">
         <v>43465</v>
       </c>
       <c r="B84" s="28" t="n">
@@ -10419,7 +10434,7 @@
         <v/>
       </c>
       <c r="G84" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C84)+0.5*COUNTIF($C$5:$C$92,C84))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C84)+(COUNTIF($C$5:$C$92,C84)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H84">
@@ -10440,7 +10455,7 @@
       </c>
       <c r="L84" s="50" t="inlineStr"/>
       <c r="M84">
-        <f>IF(F84="","",IF(F84&lt;5%,"&lt;5%",IF(F84&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F84="","",IF(F84&lt;5%,"&lt;5%",IF(F84&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N84" s="50">
@@ -10465,7 +10480,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="27" t="n">
+      <c r="A85" s="54" t="n">
         <v>43555</v>
       </c>
       <c r="B85" s="28" t="n">
@@ -10488,7 +10503,7 @@
         <v/>
       </c>
       <c r="G85" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C85)+0.5*COUNTIF($C$5:$C$92,C85))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C85)+(COUNTIF($C$5:$C$92,C85)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H85">
@@ -10509,7 +10524,7 @@
       </c>
       <c r="L85" s="50" t="inlineStr"/>
       <c r="M85">
-        <f>IF(F85="","",IF(F85&lt;5%,"&lt;5%",IF(F85&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F85="","",IF(F85&lt;5%,"&lt;5%",IF(F85&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N85" s="50">
@@ -10534,7 +10549,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="27" t="n">
+      <c r="A86" s="54" t="n">
         <v>43646</v>
       </c>
       <c r="B86" s="28" t="n">
@@ -10557,7 +10572,7 @@
         <v/>
       </c>
       <c r="G86" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C86)+0.5*COUNTIF($C$5:$C$92,C86))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C86)+(COUNTIF($C$5:$C$92,C86)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H86">
@@ -10578,7 +10593,7 @@
       </c>
       <c r="L86" s="50" t="inlineStr"/>
       <c r="M86">
-        <f>IF(F86="","",IF(F86&lt;5%,"&lt;5%",IF(F86&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F86="","",IF(F86&lt;5%,"&lt;5%",IF(F86&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N86" s="50">
@@ -10603,7 +10618,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="27" t="n">
+      <c r="A87" s="54" t="n">
         <v>43738</v>
       </c>
       <c r="B87" s="28" t="n">
@@ -10626,7 +10641,7 @@
         <v/>
       </c>
       <c r="G87" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C87)+0.5*COUNTIF($C$5:$C$92,C87))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C87)+(COUNTIF($C$5:$C$92,C87)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H87">
@@ -10647,7 +10662,7 @@
       </c>
       <c r="L87" s="50" t="inlineStr"/>
       <c r="M87">
-        <f>IF(F87="","",IF(F87&lt;5%,"&lt;5%",IF(F87&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F87="","",IF(F87&lt;5%,"&lt;5%",IF(F87&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N87" s="50">
@@ -10672,7 +10687,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="27" t="n">
+      <c r="A88" s="54" t="n">
         <v>43830</v>
       </c>
       <c r="B88" s="28" t="n">
@@ -10695,7 +10710,7 @@
         <v/>
       </c>
       <c r="G88" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C88)+0.5*COUNTIF($C$5:$C$92,C88))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C88)+(COUNTIF($C$5:$C$92,C88)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H88">
@@ -10716,7 +10731,7 @@
       </c>
       <c r="L88" s="50" t="inlineStr"/>
       <c r="M88">
-        <f>IF(F88="","",IF(F88&lt;5%,"&lt;5%",IF(F88&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F88="","",IF(F88&lt;5%,"&lt;5%",IF(F88&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N88" s="50">
@@ -10741,7 +10756,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="27" t="n">
+      <c r="A89" s="54" t="n">
         <v>43921</v>
       </c>
       <c r="B89" s="28" t="n">
@@ -10764,7 +10779,7 @@
         <v/>
       </c>
       <c r="G89" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C89)+0.5*COUNTIF($C$5:$C$92,C89))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C89)+(COUNTIF($C$5:$C$92,C89)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H89">
@@ -10785,7 +10800,7 @@
       </c>
       <c r="L89" s="50" t="inlineStr"/>
       <c r="M89">
-        <f>IF(F89="","",IF(F89&lt;5%,"&lt;5%",IF(F89&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F89="","",IF(F89&lt;5%,"&lt;5%",IF(F89&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N89" s="50">
@@ -10810,7 +10825,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="27" t="n">
+      <c r="A90" s="54" t="n">
         <v>44012</v>
       </c>
       <c r="B90" s="28" t="n">
@@ -10833,7 +10848,7 @@
         <v/>
       </c>
       <c r="G90" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C90)+0.5*COUNTIF($C$5:$C$92,C90))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C90)+(COUNTIF($C$5:$C$92,C90)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H90">
@@ -10854,7 +10869,7 @@
       </c>
       <c r="L90" s="50" t="inlineStr"/>
       <c r="M90">
-        <f>IF(F90="","",IF(F90&lt;5%,"&lt;5%",IF(F90&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F90="","",IF(F90&lt;5%,"&lt;5%",IF(F90&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N90" s="50">
@@ -10879,7 +10894,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="27" t="n">
+      <c r="A91" s="54" t="n">
         <v>44104</v>
       </c>
       <c r="B91" s="28" t="n">
@@ -10902,7 +10917,7 @@
         <v/>
       </c>
       <c r="G91" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C91)+0.5*COUNTIF($C$5:$C$92,C91))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C91)+(COUNTIF($C$5:$C$92,C91)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H91">
@@ -10923,7 +10938,7 @@
       </c>
       <c r="L91" s="50" t="inlineStr"/>
       <c r="M91">
-        <f>IF(F91="","",IF(F91&lt;5%,"&lt;5%",IF(F91&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F91="","",IF(F91&lt;5%,"&lt;5%",IF(F91&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N91" s="50">
@@ -10948,7 +10963,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="27" t="n">
+      <c r="A92" s="54" t="n">
         <v>44196</v>
       </c>
       <c r="B92" s="28" t="n">
@@ -10971,7 +10986,7 @@
         <v/>
       </c>
       <c r="G92" s="50">
-        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C92)+0.5*COUNTIF($C$5:$C$92,C92))/COUNT($C$5:$C$92),"")</f>
+        <f>IFERROR((COUNTIF($C$5:$C$92,"&lt;"&amp;C92)+(COUNTIF($C$5:$C$92,C92)+1)/2)/COUNT($C$5:$C$92),"")</f>
         <v/>
       </c>
       <c r="H92">
@@ -10992,7 +11007,7 @@
       </c>
       <c r="L92" s="50" t="inlineStr"/>
       <c r="M92">
-        <f>IF(F92="","",IF(F92&lt;5%,"&lt;5%",IF(F92&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F92="","",IF(F92&lt;5%,"&lt;5%",IF(F92&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N92" s="50">
@@ -11017,7 +11032,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="27" t="n">
+      <c r="A93" s="54" t="n">
         <v>44286</v>
       </c>
       <c r="B93" s="28" t="n">
@@ -11040,7 +11055,7 @@
         <v/>
       </c>
       <c r="G93" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C93)+0.5*COUNTIF($C$93:$C$114,C93))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C93)+(COUNTIF($C$93:$C$114,C93)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H93">
@@ -11061,7 +11076,7 @@
       </c>
       <c r="L93" s="50" t="inlineStr"/>
       <c r="M93">
-        <f>IF(F93="","",IF(F93&lt;5%,"&lt;5%",IF(F93&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F93="","",IF(F93&lt;5%,"&lt;5%",IF(F93&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N93" s="50">
@@ -11086,7 +11101,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="27" t="n">
+      <c r="A94" s="54" t="n">
         <v>44377</v>
       </c>
       <c r="B94" s="28" t="n">
@@ -11109,7 +11124,7 @@
         <v/>
       </c>
       <c r="G94" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C94)+0.5*COUNTIF($C$93:$C$114,C94))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C94)+(COUNTIF($C$93:$C$114,C94)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H94">
@@ -11130,7 +11145,7 @@
       </c>
       <c r="L94" s="50" t="inlineStr"/>
       <c r="M94">
-        <f>IF(F94="","",IF(F94&lt;5%,"&lt;5%",IF(F94&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F94="","",IF(F94&lt;5%,"&lt;5%",IF(F94&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N94" s="50">
@@ -11155,7 +11170,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="27" t="n">
+      <c r="A95" s="54" t="n">
         <v>44469</v>
       </c>
       <c r="B95" s="28" t="n">
@@ -11178,7 +11193,7 @@
         <v/>
       </c>
       <c r="G95" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C95)+0.5*COUNTIF($C$93:$C$114,C95))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C95)+(COUNTIF($C$93:$C$114,C95)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H95">
@@ -11196,7 +11211,7 @@
       <c r="K95" s="50" t="inlineStr"/>
       <c r="L95" s="50" t="inlineStr"/>
       <c r="M95">
-        <f>IF(F95="","",IF(F95&lt;5%,"&lt;5%",IF(F95&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F95="","",IF(F95&lt;5%,"&lt;5%",IF(F95&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N95" s="50">
@@ -11221,7 +11236,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="27" t="n">
+      <c r="A96" s="54" t="n">
         <v>44561</v>
       </c>
       <c r="B96" s="28" t="n">
@@ -11244,7 +11259,7 @@
         <v/>
       </c>
       <c r="G96" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C96)+0.5*COUNTIF($C$93:$C$114,C96))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C96)+(COUNTIF($C$93:$C$114,C96)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H96">
@@ -11262,7 +11277,7 @@
       <c r="K96" s="50" t="inlineStr"/>
       <c r="L96" s="50" t="inlineStr"/>
       <c r="M96">
-        <f>IF(F96="","",IF(F96&lt;5%,"&lt;5%",IF(F96&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F96="","",IF(F96&lt;5%,"&lt;5%",IF(F96&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N96" s="50">
@@ -11287,7 +11302,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="27" t="n">
+      <c r="A97" s="54" t="n">
         <v>44651</v>
       </c>
       <c r="B97" s="28" t="n">
@@ -11310,7 +11325,7 @@
         <v/>
       </c>
       <c r="G97" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C97)+0.5*COUNTIF($C$93:$C$114,C97))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C97)+(COUNTIF($C$93:$C$114,C97)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H97">
@@ -11328,7 +11343,7 @@
       <c r="K97" s="50" t="inlineStr"/>
       <c r="L97" s="50" t="inlineStr"/>
       <c r="M97">
-        <f>IF(F97="","",IF(F97&lt;5%,"&lt;5%",IF(F97&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F97="","",IF(F97&lt;5%,"&lt;5%",IF(F97&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N97" s="50">
@@ -11353,7 +11368,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="27" t="n">
+      <c r="A98" s="54" t="n">
         <v>44742</v>
       </c>
       <c r="B98" s="28" t="n">
@@ -11376,7 +11391,7 @@
         <v/>
       </c>
       <c r="G98" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C98)+0.5*COUNTIF($C$93:$C$114,C98))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C98)+(COUNTIF($C$93:$C$114,C98)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H98">
@@ -11394,7 +11409,7 @@
       <c r="K98" s="50" t="inlineStr"/>
       <c r="L98" s="50" t="inlineStr"/>
       <c r="M98">
-        <f>IF(F98="","",IF(F98&lt;5%,"&lt;5%",IF(F98&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F98="","",IF(F98&lt;5%,"&lt;5%",IF(F98&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N98" s="50">
@@ -11419,7 +11434,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="27" t="n">
+      <c r="A99" s="54" t="n">
         <v>44834</v>
       </c>
       <c r="B99" s="28" t="n">
@@ -11442,7 +11457,7 @@
         <v/>
       </c>
       <c r="G99" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C99)+0.5*COUNTIF($C$93:$C$114,C99))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C99)+(COUNTIF($C$93:$C$114,C99)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H99">
@@ -11460,7 +11475,7 @@
       <c r="K99" s="50" t="inlineStr"/>
       <c r="L99" s="50" t="inlineStr"/>
       <c r="M99">
-        <f>IF(F99="","",IF(F99&lt;5%,"&lt;5%",IF(F99&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F99="","",IF(F99&lt;5%,"&lt;5%",IF(F99&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N99" s="50">
@@ -11485,7 +11500,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="27" t="n">
+      <c r="A100" s="54" t="n">
         <v>44926</v>
       </c>
       <c r="B100" s="28" t="n">
@@ -11508,7 +11523,7 @@
         <v/>
       </c>
       <c r="G100" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C100)+0.5*COUNTIF($C$93:$C$114,C100))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C100)+(COUNTIF($C$93:$C$114,C100)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H100">
@@ -11526,7 +11541,7 @@
       <c r="K100" s="50" t="inlineStr"/>
       <c r="L100" s="50" t="inlineStr"/>
       <c r="M100">
-        <f>IF(F100="","",IF(F100&lt;5%,"&lt;5%",IF(F100&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F100="","",IF(F100&lt;5%,"&lt;5%",IF(F100&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N100" s="50">
@@ -11551,7 +11566,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="27" t="n">
+      <c r="A101" s="54" t="n">
         <v>45016</v>
       </c>
       <c r="B101" s="28" t="n">
@@ -11574,7 +11589,7 @@
         <v/>
       </c>
       <c r="G101" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C101)+0.5*COUNTIF($C$93:$C$114,C101))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C101)+(COUNTIF($C$93:$C$114,C101)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H101">
@@ -11592,7 +11607,7 @@
       <c r="K101" s="50" t="inlineStr"/>
       <c r="L101" s="50" t="inlineStr"/>
       <c r="M101">
-        <f>IF(F101="","",IF(F101&lt;5%,"&lt;5%",IF(F101&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F101="","",IF(F101&lt;5%,"&lt;5%",IF(F101&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N101" s="50">
@@ -11617,7 +11632,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="27" t="n">
+      <c r="A102" s="54" t="n">
         <v>45107</v>
       </c>
       <c r="B102" s="28" t="n">
@@ -11640,7 +11655,7 @@
         <v/>
       </c>
       <c r="G102" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C102)+0.5*COUNTIF($C$93:$C$114,C102))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C102)+(COUNTIF($C$93:$C$114,C102)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H102">
@@ -11658,7 +11673,7 @@
       <c r="K102" s="50" t="inlineStr"/>
       <c r="L102" s="50" t="inlineStr"/>
       <c r="M102">
-        <f>IF(F102="","",IF(F102&lt;5%,"&lt;5%",IF(F102&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F102="","",IF(F102&lt;5%,"&lt;5%",IF(F102&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N102" s="50">
@@ -11683,7 +11698,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="27" t="n">
+      <c r="A103" s="54" t="n">
         <v>45199</v>
       </c>
       <c r="B103" s="28" t="n">
@@ -11706,7 +11721,7 @@
         <v/>
       </c>
       <c r="G103" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C103)+0.5*COUNTIF($C$93:$C$114,C103))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C103)+(COUNTIF($C$93:$C$114,C103)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H103">
@@ -11721,7 +11736,7 @@
       <c r="K103" s="50" t="inlineStr"/>
       <c r="L103" s="50" t="inlineStr"/>
       <c r="M103">
-        <f>IF(F103="","",IF(F103&lt;5%,"&lt;5%",IF(F103&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F103="","",IF(F103&lt;5%,"&lt;5%",IF(F103&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N103" s="50">
@@ -11746,7 +11761,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="27" t="n">
+      <c r="A104" s="54" t="n">
         <v>45291</v>
       </c>
       <c r="B104" s="28" t="n">
@@ -11769,7 +11784,7 @@
         <v/>
       </c>
       <c r="G104" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C104)+0.5*COUNTIF($C$93:$C$114,C104))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C104)+(COUNTIF($C$93:$C$114,C104)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H104">
@@ -11784,7 +11799,7 @@
       <c r="K104" s="50" t="inlineStr"/>
       <c r="L104" s="50" t="inlineStr"/>
       <c r="M104">
-        <f>IF(F104="","",IF(F104&lt;5%,"&lt;5%",IF(F104&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F104="","",IF(F104&lt;5%,"&lt;5%",IF(F104&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N104" s="50">
@@ -11809,7 +11824,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="27" t="n">
+      <c r="A105" s="54" t="n">
         <v>45382</v>
       </c>
       <c r="B105" s="28" t="n">
@@ -11832,7 +11847,7 @@
         <v/>
       </c>
       <c r="G105" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C105)+0.5*COUNTIF($C$93:$C$114,C105))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C105)+(COUNTIF($C$93:$C$114,C105)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H105">
@@ -11847,7 +11862,7 @@
       <c r="K105" s="50" t="inlineStr"/>
       <c r="L105" s="50" t="inlineStr"/>
       <c r="M105">
-        <f>IF(F105="","",IF(F105&lt;5%,"&lt;5%",IF(F105&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F105="","",IF(F105&lt;5%,"&lt;5%",IF(F105&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N105" s="50">
@@ -11872,7 +11887,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="27" t="n">
+      <c r="A106" s="54" t="n">
         <v>45473</v>
       </c>
       <c r="B106" s="28" t="n">
@@ -11895,7 +11910,7 @@
         <v/>
       </c>
       <c r="G106" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C106)+0.5*COUNTIF($C$93:$C$114,C106))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C106)+(COUNTIF($C$93:$C$114,C106)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H106">
@@ -11910,7 +11925,7 @@
       <c r="K106" s="50" t="inlineStr"/>
       <c r="L106" s="50" t="inlineStr"/>
       <c r="M106">
-        <f>IF(F106="","",IF(F106&lt;5%,"&lt;5%",IF(F106&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F106="","",IF(F106&lt;5%,"&lt;5%",IF(F106&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N106" s="50">
@@ -11935,7 +11950,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="27" t="n">
+      <c r="A107" s="54" t="n">
         <v>45565</v>
       </c>
       <c r="B107" s="28" t="n">
@@ -11958,7 +11973,7 @@
         <v/>
       </c>
       <c r="G107" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C107)+0.5*COUNTIF($C$93:$C$114,C107))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C107)+(COUNTIF($C$93:$C$114,C107)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H107">
@@ -11973,7 +11988,7 @@
       <c r="K107" s="50" t="inlineStr"/>
       <c r="L107" s="50" t="inlineStr"/>
       <c r="M107">
-        <f>IF(F107="","",IF(F107&lt;5%,"&lt;5%",IF(F107&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F107="","",IF(F107&lt;5%,"&lt;5%",IF(F107&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N107" s="50">
@@ -11998,7 +12013,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="27" t="n">
+      <c r="A108" s="54" t="n">
         <v>45657</v>
       </c>
       <c r="B108" s="28" t="n">
@@ -12021,7 +12036,7 @@
         <v/>
       </c>
       <c r="G108" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C108)+0.5*COUNTIF($C$93:$C$114,C108))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C108)+(COUNTIF($C$93:$C$114,C108)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H108">
@@ -12036,7 +12051,7 @@
       <c r="K108" s="50" t="inlineStr"/>
       <c r="L108" s="50" t="inlineStr"/>
       <c r="M108">
-        <f>IF(F108="","",IF(F108&lt;5%,"&lt;5%",IF(F108&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F108="","",IF(F108&lt;5%,"&lt;5%",IF(F108&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N108" s="50">
@@ -12061,7 +12076,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="27" t="n">
+      <c r="A109" s="54" t="n">
         <v>45747</v>
       </c>
       <c r="B109" s="28" t="n">
@@ -12084,7 +12099,7 @@
         <v/>
       </c>
       <c r="G109" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C109)+0.5*COUNTIF($C$93:$C$114,C109))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C109)+(COUNTIF($C$93:$C$114,C109)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H109">
@@ -12099,7 +12114,7 @@
       <c r="K109" s="50" t="inlineStr"/>
       <c r="L109" s="50" t="inlineStr"/>
       <c r="M109">
-        <f>IF(F109="","",IF(F109&lt;5%,"&lt;5%",IF(F109&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F109="","",IF(F109&lt;5%,"&lt;5%",IF(F109&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N109" s="50">
@@ -12124,7 +12139,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="27" t="n">
+      <c r="A110" s="54" t="n">
         <v>45838</v>
       </c>
       <c r="B110" s="28" t="n">
@@ -12147,7 +12162,7 @@
         <v/>
       </c>
       <c r="G110" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C110)+0.5*COUNTIF($C$93:$C$114,C110))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C110)+(COUNTIF($C$93:$C$114,C110)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H110">
@@ -12162,7 +12177,7 @@
       <c r="K110" s="50" t="inlineStr"/>
       <c r="L110" s="50" t="inlineStr"/>
       <c r="M110">
-        <f>IF(F110="","",IF(F110&lt;5%,"&lt;5%",IF(F110&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F110="","",IF(F110&lt;5%,"&lt;5%",IF(F110&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N110" s="50">
@@ -12187,7 +12202,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="27" t="n">
+      <c r="A111" s="54" t="n">
         <v>45930</v>
       </c>
       <c r="B111" s="28" t="n">
@@ -12210,7 +12225,7 @@
         <v/>
       </c>
       <c r="G111" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C111)+0.5*COUNTIF($C$93:$C$114,C111))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C111)+(COUNTIF($C$93:$C$114,C111)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H111">
@@ -12222,7 +12237,7 @@
       <c r="K111" s="50" t="inlineStr"/>
       <c r="L111" s="50" t="inlineStr"/>
       <c r="M111">
-        <f>IF(F111="","",IF(F111&lt;5%,"&lt;5%",IF(F111&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F111="","",IF(F111&lt;5%,"&lt;5%",IF(F111&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N111" s="50">
@@ -12247,7 +12262,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="27" t="n">
+      <c r="A112" s="54" t="n">
         <v>46022</v>
       </c>
       <c r="B112" s="28" t="n">
@@ -12270,7 +12285,7 @@
         <v/>
       </c>
       <c r="G112" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C112)+0.5*COUNTIF($C$93:$C$114,C112))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C112)+(COUNTIF($C$93:$C$114,C112)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H112">
@@ -12282,7 +12297,7 @@
       <c r="K112" s="50" t="inlineStr"/>
       <c r="L112" s="50" t="inlineStr"/>
       <c r="M112">
-        <f>IF(F112="","",IF(F112&lt;5%,"&lt;5%",IF(F112&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F112="","",IF(F112&lt;5%,"&lt;5%",IF(F112&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N112" s="50">
@@ -12307,7 +12322,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="27" t="n">
+      <c r="A113" s="54" t="n">
         <v>46112</v>
       </c>
       <c r="B113" s="28" t="n">
@@ -12330,7 +12345,7 @@
         <v/>
       </c>
       <c r="G113" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C113)+0.5*COUNTIF($C$93:$C$114,C113))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C113)+(COUNTIF($C$93:$C$114,C113)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H113">
@@ -12342,7 +12357,7 @@
       <c r="K113" s="50" t="inlineStr"/>
       <c r="L113" s="50" t="inlineStr"/>
       <c r="M113">
-        <f>IF(F113="","",IF(F113&lt;5%,"&lt;5%",IF(F113&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F113="","",IF(F113&lt;5%,"&lt;5%",IF(F113&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N113" s="50">
@@ -12367,7 +12382,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="27" t="n">
+      <c r="A114" s="54" t="n">
         <v>46203</v>
       </c>
       <c r="B114" s="28" t="n">
@@ -12390,7 +12405,7 @@
         <v/>
       </c>
       <c r="G114" s="50">
-        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C114)+0.5*COUNTIF($C$93:$C$114,C114))/COUNT($C$93:$C$114),"")</f>
+        <f>IFERROR((COUNTIF($C$93:$C$114,"&lt;"&amp;C114)+(COUNTIF($C$93:$C$114,C114)+1)/2)/COUNT($C$93:$C$114),"")</f>
         <v/>
       </c>
       <c r="H114">
@@ -12402,7 +12417,7 @@
       <c r="K114" s="50" t="inlineStr"/>
       <c r="L114" s="50" t="inlineStr"/>
       <c r="M114">
-        <f>IF(F114="","",IF(F114&lt;5%,"&lt;5%",IF(F114&lt;15%,"5-15%","&gt;15%")))</f>
+        <f>IF(F114="","",IF(F114&lt;5%,"&lt;5%",IF(F114&lt;=15%,"5-15%","&gt;15%")))</f>
         <v/>
       </c>
       <c r="N114" s="50">

</xml_diff>

<commit_message>
Index valuation and backtest update
</commit_message>
<xml_diff>
--- a/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
+++ b/NIFTY_Valuation_Backtest_Live_Tracker.xlsx
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;[Red](#,##0.00);-"/>
     <numFmt numFmtId="166" formatCode="0.00x;[Red](0.00x);-"/>
@@ -36,6 +36,7 @@
     <numFmt numFmtId="170" formatCode="0.0x;[Red](0.0x);-"/>
     <numFmt numFmtId="171" formatCode="0.00x"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -2423,7 +2424,7 @@
         </is>
       </c>
       <c r="B5" s="42" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="D5" s="6">
         <f>B20</f>
@@ -2437,7 +2438,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>23346.4</v>
+        <v>23414.3</v>
       </c>
     </row>
     <row r="7">
@@ -2447,7 +2448,7 @@
         </is>
       </c>
       <c r="B7" s="43" t="n">
-        <v>19.74</v>
+        <v>19.79</v>
       </c>
     </row>
     <row r="8">
@@ -2505,7 +2506,7 @@
         </is>
       </c>
       <c r="B12" s="42" t="n">
-        <v>45918</v>
+        <v>45919</v>
       </c>
     </row>
     <row r="13">
@@ -2515,7 +2516,7 @@
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>25423.6</v>
+        <v>25327.05</v>
       </c>
     </row>
     <row r="14">
@@ -2525,7 +2526,7 @@
         </is>
       </c>
       <c r="B14" s="47" t="n">
-        <v>22.33</v>
+        <v>22.25</v>
       </c>
     </row>
     <row r="15">
@@ -13687,10 +13688,10 @@
     </row>
     <row r="70">
       <c r="A70" s="54" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="B70" s="57" t="n">
-        <v>19.74</v>
+        <v>19.79</v>
       </c>
       <c r="C70" s="30" t="inlineStr">
         <is>
@@ -13721,7 +13722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13907,6 +13908,50 @@
       <c r="L6" s="4" t="inlineStr">
         <is>
           <t>https://nsearchives.nseindia.com/content/indices/ind_close_all_18092026.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="58" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B7" s="59" t="n">
+        <v>23414.3</v>
+      </c>
+      <c r="C7" s="60" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="D7" s="65" t="n">
+        <v>0.05303030303030303</v>
+      </c>
+      <c r="E7" s="62" t="n">
+        <v>1183.137948458818</v>
+      </c>
+      <c r="F7" s="65" t="n">
+        <v>0.03939540346028036</v>
+      </c>
+      <c r="G7" s="63" t="n">
+        <v>94.6969696969697</v>
+      </c>
+      <c r="H7" s="63" t="n">
+        <v>35.75816138411214</v>
+      </c>
+      <c r="I7" s="63" t="n">
+        <v>77.01532720311242</v>
+      </c>
+      <c r="J7" s="64" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/indices/ind_close_all_21092026.csv</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/indices/ind_close_all_21092026.csv</t>
         </is>
       </c>
     </row>

</xml_diff>